<commit_message>
Daily NSE automation update
</commit_message>
<xml_diff>
--- a/exports/securities_below_20_2026-05-19.xlsx
+++ b/exports/securities_below_20_2026-05-19.xlsx
@@ -476,22 +476,22 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>5.04</t>
+          <t>5.00</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>17.76</t>
+          <t>16.82</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>10,15,676</t>
+          <t>10,66,304</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>50.07</t>
+          <t>52.57</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -528,22 +528,22 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>12.52</t>
+          <t>12.51</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>9.92</t>
+          <t>9.83</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2,31,559</t>
+          <t>2,41,316</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>28.74</t>
+          <t>29.95</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -555,104 +555,104 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TPHQ</t>
+          <t>MANUGRAPH</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.51</t>
+          <t>13.41</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.54</t>
+          <t>13.84</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.50</t>
+          <t>13.25</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0.50</t>
+          <t>12.93</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.53</t>
+          <t>13.72</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>6.00</t>
+          <t>6.11</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>8,11,906</t>
+          <t>4,180</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>4.22</t>
+          <t>0.56</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>17-Sep-2024</t>
+          <t>20-Sep-2024</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MANUGRAPH</t>
+          <t>TPHQ</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>13.41</t>
+          <t>0.51</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>13.74</t>
+          <t>0.54</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>13.25</t>
+          <t>0.50</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12.93</t>
+          <t>0.50</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>13.68</t>
+          <t>0.53</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>5.80</t>
+          <t>6.00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>4,028</t>
+          <t>8,24,110</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>0.54</t>
+          <t>4.29</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>20-Sep-2024</t>
+          <t>17-Sep-2024</t>
         </is>
       </c>
     </row>
@@ -694,12 +694,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1,97,624</t>
+          <t>1,98,988</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>23.97</t>
+          <t>24.14</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -746,12 +746,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>79,233</t>
+          <t>81,714</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>7.28</t>
+          <t>7.51</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -850,12 +850,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>77,379</t>
+          <t>77,479</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>7.04</t>
+          <t>7.05</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -867,203 +867,203 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>VCL</t>
+          <t>KSHITIJPOL</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1.43</t>
+          <t>3.56</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1.50</t>
+          <t>3.92</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>3.56</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.43</t>
+          <t>3.74</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>1.50</t>
+          <t>3.92</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>4.90</t>
+          <t>4.81</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2,15,861</t>
+          <t>10,03,879</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>3.17</t>
+          <t>36.94</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>19-Sep-2024</t>
+          <t>18-Jun-2024</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SVPGLOB</t>
+          <t>KHANDSE</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>3.68</t>
+          <t>18.90</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>3.88</t>
+          <t>18.90</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>3.55</t>
+          <t>17.00</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>3.70</t>
+          <t>16.97</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>3.88</t>
+          <t>17.78</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>4.86</t>
+          <t>4.77</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>54,633</t>
+          <t>9,349</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2.11</t>
+          <t>1.71</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>20-Sep-2024</t>
+          <t>19-Sep-2024</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>KSHITIJPOL</t>
+          <t>GTLINFRA</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>3.56</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3.92</t>
+          <t>1.35</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>3.56</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>3.74</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>3.92</t>
+          <t>1.35</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>4.81</t>
+          <t>4.65</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>9,84,215</t>
+          <t>2,33,74,375</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>36.22</t>
+          <t>306.20</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>18-Jun-2024</t>
+          <t>21-Sep-2015</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>KHANDSE</t>
+          <t>PNC</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>18.90</t>
+          <t>19.10</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>18.90</t>
+          <t>19.90</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>17.00</t>
+          <t>18.15</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>16.97</t>
+          <t>19.01</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>17.78</t>
+          <t>19.89</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>4.77</t>
+          <t>4.63</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>9,349</t>
+          <t>1,620</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>1.71</t>
+          <t>0.31</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1075,151 +1075,151 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>GTLINFRA</t>
+          <t>SHYAMCENT</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>4.98</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.35</t>
+          <t>5.45</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>4.57</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>4.97</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1.35</t>
+          <t>5.20</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>4.65</t>
+          <t>4.63</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2,16,90,954</t>
+          <t>89,361</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>284.15</t>
+          <t>4.58</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>21-Sep-2015</t>
+          <t>19-Sep-2024</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SHYAMCENT</t>
+          <t>FILATFASH</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>4.98</t>
+          <t>0.23</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>5.45</t>
+          <t>0.24</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>4.57</t>
+          <t>0.23</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>4.97</t>
+          <t>0.23</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>5.19</t>
+          <t>0.24</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>4.43</t>
+          <t>4.35</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>89,261</t>
+          <t>65,91,612</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>4.57</t>
+          <t>15.16</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>19-Sep-2024</t>
+          <t>20-Sep-2024</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>FILATFASH</t>
+          <t>ROLLT</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0.23</t>
+          <t>2.07</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.24</t>
+          <t>2.18</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.23</t>
+          <t>1.99</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>0.23</t>
+          <t>2.08</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>0.24</t>
+          <t>2.17</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>4.35</t>
+          <t>4.33</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>63,39,729</t>
+          <t>2,93,109</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>14.58</t>
+          <t>6.27</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1266,12 +1266,12 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>19,18,020</t>
+          <t>19,29,630</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>32.61</t>
+          <t>32.80</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1283,156 +1283,156 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>AKG</t>
+          <t>JYOTISTRUC</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11.04</t>
+          <t>12.10</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>11.70</t>
+          <t>12.69</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>11.04</t>
+          <t>12.05</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>11.06</t>
+          <t>12.10</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>11.53</t>
+          <t>12.60</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>4.25</t>
+          <t>4.13</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>3,396</t>
+          <t>30,18,054</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>0.39</t>
+          <t>371.52</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>17-Sep-2024</t>
+          <t>10-Feb-2025</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>JYOTISTRUC</t>
+          <t>ASHOKAMET</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>12.10</t>
+          <t>15.90</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>12.69</t>
+          <t>16.60</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>12.05</t>
+          <t>15.80</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>12.10</t>
+          <t>15.66</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>12.60</t>
+          <t>16.30</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>4.13</t>
+          <t>4.09</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>27,52,233</t>
+          <t>9,253</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>338.25</t>
+          <t>1.49</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>10-Feb-2025</t>
+          <t>06-Sep-2024</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>HAVISHA</t>
+          <t>NEXTMEDIA</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1.49</t>
+          <t>4.01</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1.58</t>
+          <t>4.17</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1.49</t>
+          <t>3.98</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.52</t>
+          <t>4.01</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>1.58</t>
+          <t>4.17</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>3.95</t>
+          <t>3.99</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1,231</t>
+          <t>9,638</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>0.02</t>
+          <t>0.38</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>17-Sep-2024</t>
+          <t>22-Aug-2017</t>
         </is>
       </c>
     </row>
@@ -1474,12 +1474,12 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>58,20,311</t>
+          <t>58,79,196</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>30.85</t>
+          <t>31.16</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1526,12 +1526,12 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>5,48,479</t>
+          <t>5,60,320</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>23.53</t>
+          <t>24.04</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1578,12 +1578,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1,34,099</t>
+          <t>1,58,949</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>6.54</t>
+          <t>7.76</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1682,12 +1682,12 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>34,819</t>
+          <t>41,626</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>1.60</t>
+          <t>1.91</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1699,307 +1699,307 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>EUROTEXIND</t>
+          <t>ASTRON</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>15.56</t>
+          <t>4.19</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>15.91</t>
+          <t>4.20</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>15.56</t>
+          <t>4.03</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>16.09</t>
+          <t>4.20</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>15.58</t>
+          <t>4.03</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>-3.17</t>
+          <t>-4.05</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1,324</t>
+          <t>11,824</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>0.21</t>
+          <t>0.48</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>12-Sep-2024</t>
+          <t>23-Sep-2024</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>VIVIMEDLAB</t>
+          <t>DPSCLTD</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>6.30</t>
+          <t>9.71</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>6.50</t>
+          <t>9.87</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>6.10</t>
+          <t>9.42</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>6.32</t>
+          <t>9.94</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>6.14</t>
+          <t>9.57</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>-2.85</t>
+          <t>-3.72</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1,01,686</t>
+          <t>1,44,430</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>6.29</t>
+          <t>13.88</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>27-Dec-2024</t>
+          <t>12-Sep-2025</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>DPSCLTD</t>
+          <t>EUROTEXIND</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>9.71</t>
+          <t>15.56</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>9.87</t>
+          <t>15.91</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>9.42</t>
+          <t>15.56</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>9.94</t>
+          <t>16.09</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>9.67</t>
+          <t>15.58</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>-2.72</t>
+          <t>-3.17</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1,42,916</t>
+          <t>1,324</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>13.73</t>
+          <t>0.21</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>12-Sep-2025</t>
+          <t>12-Sep-2024</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>RADAAN</t>
+          <t>TIJARIA</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>3.20</t>
+          <t>4.72</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>3.20</t>
+          <t>4.93</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2.92</t>
+          <t>4.60</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>3.06</t>
+          <t>4.71</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>3.00</t>
+          <t>4.60</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>-1.96</t>
+          <t>-2.34</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1,249</t>
+          <t>17,358</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>0.04</t>
+          <t>0.85</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>23-Sep-2022</t>
+          <t>19-Sep-2024</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SEYAIND</t>
+          <t>AIRAN</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>15.05</t>
+          <t>16.27</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>15.05</t>
+          <t>16.93</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>15.05</t>
+          <t>16.25</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>15.35</t>
+          <t>16.67</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>15.05</t>
+          <t>16.29</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>-1.95</t>
+          <t>-2.28</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>4,095</t>
+          <t>16,356</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>0.62</t>
+          <t>2.68</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>17-Dec-2020</t>
+          <t>14-Aug-2019</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>MADHUCON</t>
+          <t>AKI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>5.70</t>
+          <t>4.79</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>5.99</t>
+          <t>4.99</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>5.60</t>
+          <t>4.70</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>5.71</t>
+          <t>4.80</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>5.60</t>
+          <t>4.70</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>-1.93</t>
+          <t>-2.08</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1,316</t>
+          <t>19,411</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>0.08</t>
+          <t>0.93</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2011,416 +2011,416 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>GVKPIL</t>
+          <t>SEYAIND</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>3.08</t>
+          <t>15.05</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>3.08</t>
+          <t>15.05</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>3.08</t>
+          <t>15.05</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>3.14</t>
+          <t>15.35</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>3.08</t>
+          <t>15.05</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>-1.91</t>
+          <t>-1.95</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1,75,201</t>
+          <t>4,105</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>5.40</t>
+          <t>0.62</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>27-Dec-2024</t>
+          <t>17-Dec-2020</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ALOKINDS</t>
+          <t>MADHUCON</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>13.22</t>
+          <t>5.70</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>13.29</t>
+          <t>5.99</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>12.85</t>
+          <t>5.60</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>13.18</t>
+          <t>5.71</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>12.93</t>
+          <t>5.60</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>-1.90</t>
+          <t>-1.93</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>30,71,964</t>
+          <t>1,316</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>398.74</t>
+          <t>0.08</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>20-Sep-2024</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ACCURACY</t>
+          <t>GVKPIL</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>5.44</t>
+          <t>3.08</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
+          <t>3.08</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>3.08</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>3.14</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>3.08</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>-1.91</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>1,78,118</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
           <t>5.49</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>5.27</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>5.46</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>5.36</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>-1.83</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>74,251</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>3.94</t>
-        </is>
-      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>15-Feb-2023</t>
+          <t>27-Dec-2024</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SUVIDHAA</t>
+          <t>RNBDENIMS</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>3.03</t>
+          <t>11.62</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>3.03</t>
+          <t>11.99</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2.88</t>
+          <t>11.28</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2.93</t>
+          <t>11.62</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2.88</t>
+          <t>11.40</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>-1.71</t>
+          <t>-1.89</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>16,204</t>
+          <t>2,25,209</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>0.47</t>
+          <t>26.08</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>23-Sep-2024</t>
+          <t>02-Apr-2026</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>LAL</t>
+          <t>DISHTV</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>7.14</t>
+          <t>3.15</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>7.20</t>
+          <t>3.21</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>6.91</t>
+          <t>3.10</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>7.14</t>
+          <t>3.20</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>7.02</t>
+          <t>3.14</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>-1.68</t>
+          <t>-1.88</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>1,697</t>
+          <t>7,38,244</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>0.12</t>
+          <t>23.11</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>23-Sep-2024</t>
+          <t>05-Nov-2018</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>GLOBE</t>
+          <t>CREATIVEYE</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2.38</t>
+          <t>6.98</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2.44</t>
+          <t>7.04</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2.38</t>
+          <t>6.76</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2.44</t>
+          <t>6.99</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2.40</t>
+          <t>6.86</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>-1.64</t>
+          <t>-1.86</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>35,460</t>
+          <t>4,223</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>0.86</t>
+          <t>0.29</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>17-Jan-2025</t>
+          <t>23-Sep-2024</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>IBULLSLTD</t>
+          <t>SHAH</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>17.53</t>
+          <t>5.49</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>18.75</t>
+          <t>5.49</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>17.53</t>
+          <t>5.31</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>18.45</t>
+          <t>5.41</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>18.16</t>
+          <t>5.31</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>-1.57</t>
+          <t>-1.85</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>11,15,046</t>
+          <t>1,56,188</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>200.71</t>
+          <t>8.42</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>19-Sep-2024</t>
+          <t>04-May-2023</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>DISHTV</t>
+          <t>ACCURACY</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>3.15</t>
+          <t>5.44</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>3.21</t>
+          <t>5.49</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>3.10</t>
+          <t>5.27</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>3.20</t>
+          <t>5.46</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>3.15</t>
+          <t>5.36</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>-1.56</t>
+          <t>-1.83</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>7,21,945</t>
+          <t>74,272</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>22.60</t>
+          <t>3.94</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>05-Nov-2018</t>
+          <t>15-Feb-2023</t>
         </is>
       </c>
     </row>
@@ -2452,22 +2452,22 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>13.93</t>
+          <t>13.90</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>-1.49</t>
+          <t>-1.70</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>11,275</t>
+          <t>11,846</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>1.59</t>
+          <t>1.67</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -2479,42 +2479,42 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>INFOMEDIA</t>
+          <t>CINEVISTA</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>5.33</t>
+          <t>16.20</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>6.00</t>
+          <t>16.44</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>5.33</t>
+          <t>15.70</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>5.69</t>
+          <t>16.20</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>5.61</t>
+          <t>15.93</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>-1.41</t>
+          <t>-1.67</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>3,413</t>
+          <t>1,245</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2524,7 +2524,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>10-Aug-2018</t>
+          <t>13-Sep-2024</t>
         </is>
       </c>
     </row>

</xml_diff>